<commit_message>
Commit Final de Practica
</commit_message>
<xml_diff>
--- a/Test 2/Permisosasignados202604161635_3080bca9-550a-4ced-ab00-fadfb4fdf81c.xlsx
+++ b/Test 2/Permisosasignados202604161635_3080bca9-550a-4ced-ab00-fadfb4fdf81c.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://femcom-my.sharepoint.com/personal/maximiliano_sanpedro_oxxo_com/Documents/Documentos/GitHub/Practica-Oxxo/Test 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_78C8E37254527A566A800CC01E8324448101459A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93C173E6-BED5-4419-8A72-21D6474B4E21}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_78C8E37254527A566A800CC01E8324448101459A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1901130-B080-4DF4-A219-3DA2D3550107}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="7215" yWindow="5940" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Content!$C$1:$C$210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Content!$A$1:$N$210</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2828,6 +2828,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11652,7 +11656,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C210" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:N210" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 OXXO | Uso Interno</oddFooter>

</xml_diff>